<commit_message>
Update ingestion flow and statistics/cache improvements
</commit_message>
<xml_diff>
--- a/mts/DP2-PMSR.xlsx
+++ b/mts/DP2-PMSR.xlsx
@@ -129,7 +129,7 @@
     <t>prov:endedAtTime</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821864</t>
+    <t>pmsr:DPL1784614821864</t>
   </si>
   <si>
     <t>vstoi:Deployment</t>
@@ -150,7 +150,7 @@
     <t>2025-06-05T13:01:02.000</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821865</t>
+    <t>pmsr:DPL1784614821865</t>
   </si>
   <si>
     <t>ASL 5000TM Lung Solution SN:010002 at ESSCVP Lisboa Main Simulation Room</t>
@@ -159,7 +159,7 @@
     <t>pmsr:INI1784603367298</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821866</t>
+    <t>pmsr:DPL1784614821866</t>
   </si>
   <si>
     <t>EMS-MAN (Emergency Medical Skills)–Adult Male-Simbodies SN:010003 at ESSCVP Lisboa Main Simulation Room</t>
@@ -168,7 +168,7 @@
     <t>pmsr:INI1784603367299</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821867</t>
+    <t>pmsr:DPL1784614821867</t>
   </si>
   <si>
     <t>EMS-T Trainer (Emergency Medical Skills – Torso Trainer) SN:010004 at ESSCVP Lisboa Main Simulation Room</t>
@@ -177,7 +177,7 @@
     <t>pmsr:INI1784603367301</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821868</t>
+    <t>pmsr:DPL1784614821868</t>
   </si>
   <si>
     <t>HEART WORKS SN:010005 at ESSCVP Lisboa Main Simulation Room</t>
@@ -186,7 +186,7 @@
     <t>pmsr:INI1784603367302</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821869</t>
+    <t>pmsr:DPL1784614821869</t>
   </si>
   <si>
     <t>Hybrids VITA SN:010006 at ESSCVP Lisboa Main Simulation Room</t>
@@ -195,7 +195,7 @@
     <t>pmsr:INI1784603367303</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821870</t>
+    <t>pmsr:DPL1784614821870</t>
   </si>
   <si>
     <t>SimCapture Enterprise Cloud (Subscrição Anual) SN:010007 at ESSCVP Lisboa Main Simulation Room</t>
@@ -204,7 +204,7 @@
     <t>pmsr:INI1784603367305</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821871</t>
+    <t>pmsr:DPL1784614821871</t>
   </si>
   <si>
     <t>Simulador de Ressonância Magnética:Corsmed SN:010008 at ESSCVP Lisboa Main Simulation Room</t>
@@ -213,7 +213,7 @@
     <t>pmsr:INI1784603367306</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821872</t>
+    <t>pmsr:DPL1784614821872</t>
   </si>
   <si>
     <t>Simulador pediátrico- SimJunior  SN:010009 at ESSCVP Lisboa Main Simulation Room</t>
@@ -222,7 +222,7 @@
     <t>pmsr:INI1784603367307</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821873</t>
+    <t>pmsr:DPL1784614821873</t>
   </si>
   <si>
     <t>Simulador SiMmom SN:010010 at ESSCVP Lisboa Main Simulation Room</t>
@@ -231,7 +231,7 @@
     <t>pmsr:INI1784603367308</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821874</t>
+    <t>pmsr:DPL1784614821874</t>
   </si>
   <si>
     <t>Sistema de Gestão do Centro de Simulação Laerdal SimCapture SN:010011 at ESSCVP Lisboa Main Simulation Room</t>
@@ -240,7 +240,7 @@
     <t>pmsr:INI1784603367310</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821875</t>
+    <t>pmsr:DPL1784614821875</t>
   </si>
   <si>
     <t>Braços de Punção SN:020001 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -252,7 +252,7 @@
     <t>pmsr:INI1784603367311</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821876</t>
+    <t>pmsr:DPL1784614821876</t>
   </si>
   <si>
     <t>Camara de Learning Space SN:020002 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -261,7 +261,7 @@
     <t>pmsr:INI1784603367312</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821877</t>
+    <t>pmsr:DPL1784614821877</t>
   </si>
   <si>
     <t>Ecógrafos/Sonda Butterfly SN:020003 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -270,7 +270,7 @@
     <t>pmsr:INI1784603367314</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821878</t>
+    <t>pmsr:DPL1784614821878</t>
   </si>
   <si>
     <t>Manequim de Alta Fidelidade SN:020004 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -279,7 +279,7 @@
     <t>pmsr:INI1784603367315</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821879</t>
+    <t>pmsr:DPL1784614821879</t>
   </si>
   <si>
     <t>Medidor de pressão respiratória microRPM SN:020005 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -288,7 +288,7 @@
     <t>pmsr:INI1784603367316</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821880</t>
+    <t>pmsr:DPL1784614821880</t>
   </si>
   <si>
     <t>Quadro interativo com suporte (horizontal e vertical) SN:020006 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -297,7 +297,7 @@
     <t>pmsr:INI1784603367318</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821881</t>
+    <t>pmsr:DPL1784614821881</t>
   </si>
   <si>
     <t>Simulador de punção arterial SN:020007 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -306,7 +306,7 @@
     <t>pmsr:INI1784603367319</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821882</t>
+    <t>pmsr:DPL1784614821882</t>
   </si>
   <si>
     <t>Tablet SN:020008 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -315,7 +315,7 @@
     <t>pmsr:INI1784603367320</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821883</t>
+    <t>pmsr:DPL1784614821883</t>
   </si>
   <si>
     <t>Tablet SN:020009 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -324,7 +324,7 @@
     <t>pmsr:INI1784603367322</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821884</t>
+    <t>pmsr:DPL1784614821884</t>
   </si>
   <si>
     <t>Tablet SN:020010 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -333,7 +333,7 @@
     <t>pmsr:INI1784603367323</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821885</t>
+    <t>pmsr:DPL1784614821885</t>
   </si>
   <si>
     <t>Tablet SN:020011 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -342,7 +342,7 @@
     <t>pmsr:INI1784603367324</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821886</t>
+    <t>pmsr:DPL1784614821886</t>
   </si>
   <si>
     <t>Tablet SN:020012 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -351,7 +351,7 @@
     <t>pmsr:INI1784603367325</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821887</t>
+    <t>pmsr:DPL1784614821887</t>
   </si>
   <si>
     <t>Tablet SN:020013 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -360,7 +360,7 @@
     <t>pmsr:INI1784603367327</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821888</t>
+    <t>pmsr:DPL1784614821888</t>
   </si>
   <si>
     <t>Tablet SN:020014 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -369,7 +369,7 @@
     <t>pmsr:INI1784603367328</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821889</t>
+    <t>pmsr:DPL1784614821889</t>
   </si>
   <si>
     <t>Tablet SN:020015 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -378,7 +378,7 @@
     <t>pmsr:INI1784603367329</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821890</t>
+    <t>pmsr:DPL1784614821890</t>
   </si>
   <si>
     <t>Tablet SN:020016 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -387,7 +387,7 @@
     <t>pmsr:INI1784603367331</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821891</t>
+    <t>pmsr:DPL1784614821891</t>
   </si>
   <si>
     <t>Tablet SN:020017 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -396,7 +396,7 @@
     <t>pmsr:INI1784603367332</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821892</t>
+    <t>pmsr:DPL1784614821892</t>
   </si>
   <si>
     <t>Tablet SN:020018 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -405,7 +405,7 @@
     <t>pmsr:INI1784603367333</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821893</t>
+    <t>pmsr:DPL1784614821893</t>
   </si>
   <si>
     <t>Tablet SN:020019 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -414,7 +414,7 @@
     <t>pmsr:INI1784603367335</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821894</t>
+    <t>pmsr:DPL1784614821894</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020020 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -423,7 +423,7 @@
     <t>pmsr:INI1784603367336</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821895</t>
+    <t>pmsr:DPL1784614821895</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020021 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -432,7 +432,7 @@
     <t>pmsr:INI1784603367337</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821896</t>
+    <t>pmsr:DPL1784614821896</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020022 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -441,7 +441,7 @@
     <t>pmsr:INI1784603367339</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821897</t>
+    <t>pmsr:DPL1784614821897</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020023 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -450,7 +450,7 @@
     <t>pmsr:INI1784603367340</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821898</t>
+    <t>pmsr:DPL1784614821898</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020024 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -459,7 +459,7 @@
     <t>pmsr:INI1784603367341</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821899</t>
+    <t>pmsr:DPL1784614821899</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020025 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -468,7 +468,7 @@
     <t>pmsr:INI1784603367343</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821900</t>
+    <t>pmsr:DPL1784614821900</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020026 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -477,7 +477,7 @@
     <t>pmsr:INI1784603367344</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821901</t>
+    <t>pmsr:DPL1784614821901</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020027 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -486,7 +486,7 @@
     <t>pmsr:INI1784603367345</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821902</t>
+    <t>pmsr:DPL1784614821902</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020028 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -495,7 +495,7 @@
     <t>pmsr:INI1784603367346</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821903</t>
+    <t>pmsr:DPL1784614821903</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020029 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -504,7 +504,7 @@
     <t>pmsr:INI1784603367348</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821904</t>
+    <t>pmsr:DPL1784614821904</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020030 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -513,7 +513,7 @@
     <t>pmsr:INI1784603367349</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821905</t>
+    <t>pmsr:DPL1784614821905</t>
   </si>
   <si>
     <t>Óculos de Realidade Virtual SN:020031 at ESSCVP Olivais Azambuja Main Simulation Room</t>
@@ -522,7 +522,7 @@
     <t>pmsr:INI1784603367350</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821906</t>
+    <t>pmsr:DPL1784614821906</t>
   </si>
   <si>
     <t>Camara 360º OWL (suporte teto) SN:030001 at UA Main Simulation Room</t>
@@ -534,7 +534,7 @@
     <t>pmsr:INI1784603367352</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821907</t>
+    <t>pmsr:DPL1784614821907</t>
   </si>
   <si>
     <t>Câmara Video Canon R7 SN:030002 at UA Main Simulation Room</t>
@@ -543,7 +543,7 @@
     <t>pmsr:INI1784603367353</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821908</t>
+    <t>pmsr:DPL1784614821908</t>
   </si>
   <si>
     <t>DJI Mic duplo lapela WIFI SN:030003 at UA Main Simulation Room</t>
@@ -552,7 +552,7 @@
     <t>pmsr:INI1784603367354</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821909</t>
+    <t>pmsr:DPL1784614821909</t>
   </si>
   <si>
     <t>Emissor Video Wireless Hollyland Mars 4K SN:030004 at UA Main Simulation Room</t>
@@ -561,7 +561,7 @@
     <t>pmsr:INI1784603367356</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821910</t>
+    <t>pmsr:DPL1784614821910</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030005 at UA Main Simulation Room</t>
@@ -570,7 +570,7 @@
     <t>pmsr:INI1784603367357</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821911</t>
+    <t>pmsr:DPL1784614821911</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030006 at UA Main Simulation Room</t>
@@ -579,7 +579,7 @@
     <t>pmsr:INI1784603367358</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821912</t>
+    <t>pmsr:DPL1784614821912</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030007 at UA Main Simulation Room</t>
@@ -588,7 +588,7 @@
     <t>pmsr:INI1784603367360</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821913</t>
+    <t>pmsr:DPL1784614821913</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030008 at UA Main Simulation Room</t>
@@ -597,7 +597,7 @@
     <t>pmsr:INI1784603367361</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821914</t>
+    <t>pmsr:DPL1784614821914</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030009 at UA Main Simulation Room</t>
@@ -606,7 +606,7 @@
     <t>pmsr:INI1784603367362</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821915</t>
+    <t>pmsr:DPL1784614821915</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030010 at UA Main Simulation Room</t>
@@ -615,7 +615,7 @@
     <t>pmsr:INI1784603367363</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821916</t>
+    <t>pmsr:DPL1784614821916</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030011 at UA Main Simulation Room</t>
@@ -624,7 +624,7 @@
     <t>pmsr:INI1784603367365</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821917</t>
+    <t>pmsr:DPL1784614821917</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030012 at UA Main Simulation Room</t>
@@ -633,7 +633,7 @@
     <t>pmsr:INI1784603367366</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821918</t>
+    <t>pmsr:DPL1784614821918</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030013 at UA Main Simulation Room</t>
@@ -642,7 +642,7 @@
     <t>pmsr:INI1784603367367</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821919</t>
+    <t>pmsr:DPL1784614821919</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030014 at UA Main Simulation Room</t>
@@ -651,7 +651,7 @@
     <t>pmsr:INI1784603367369</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821920</t>
+    <t>pmsr:DPL1784614821920</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030015 at UA Main Simulation Room</t>
@@ -660,7 +660,7 @@
     <t>pmsr:INI1784603367370</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821921</t>
+    <t>pmsr:DPL1784614821921</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030016 at UA Main Simulation Room</t>
@@ -669,7 +669,7 @@
     <t>pmsr:INI1784603367371</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821922</t>
+    <t>pmsr:DPL1784614821922</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030017 at UA Main Simulation Room</t>
@@ -678,7 +678,7 @@
     <t>pmsr:INI1784603367373</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821923</t>
+    <t>pmsr:DPL1784614821923</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030018 at UA Main Simulation Room</t>
@@ -687,7 +687,7 @@
     <t>pmsr:INI1784603367374</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821924</t>
+    <t>pmsr:DPL1784614821924</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030019 at UA Main Simulation Room</t>
@@ -696,7 +696,7 @@
     <t>pmsr:INI1784603367375</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821925</t>
+    <t>pmsr:DPL1784614821925</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030020 at UA Main Simulation Room</t>
@@ -705,7 +705,7 @@
     <t>pmsr:INI1784603367377</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821926</t>
+    <t>pmsr:DPL1784614821926</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030021 at UA Main Simulation Room</t>
@@ -714,7 +714,7 @@
     <t>pmsr:INI1784603367378</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821927</t>
+    <t>pmsr:DPL1784614821927</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030022 at UA Main Simulation Room</t>
@@ -723,7 +723,7 @@
     <t>pmsr:INI1784603367379</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821928</t>
+    <t>pmsr:DPL1784614821928</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030023 at UA Main Simulation Room</t>
@@ -732,7 +732,7 @@
     <t>pmsr:INI1784603367381</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821929</t>
+    <t>pmsr:DPL1784614821929</t>
   </si>
   <si>
     <t>Estação de trabalho base SN:030024 at UA Main Simulation Room</t>
@@ -741,7 +741,7 @@
     <t>pmsr:INI1784603367382</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821930</t>
+    <t>pmsr:DPL1784614821930</t>
   </si>
   <si>
     <t>Lente Câmara SN:030025 at UA Main Simulation Room</t>
@@ -750,7 +750,7 @@
     <t>pmsr:INI1784603367383</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821931</t>
+    <t>pmsr:DPL1784614821931</t>
   </si>
   <si>
     <t>Matriz video HDMI (4 saidas) SN:030026 at UA Main Simulation Room</t>
@@ -759,7 +759,7 @@
     <t>pmsr:INI1784603367384</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821932</t>
+    <t>pmsr:DPL1784614821932</t>
   </si>
   <si>
     <t>Monitores 27" 4K SN:030027 at UA Main Simulation Room</t>
@@ -768,7 +768,7 @@
     <t>pmsr:INI1784603367386</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821933</t>
+    <t>pmsr:DPL1784614821933</t>
   </si>
   <si>
     <t>Monitores 27" 4K SN:030028 at UA Main Simulation Room</t>
@@ -777,7 +777,7 @@
     <t>pmsr:INI1784603367387</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821934</t>
+    <t>pmsr:DPL1784614821934</t>
   </si>
   <si>
     <t>Portátil Workstation SN:030029 at UA Main Simulation Room</t>
@@ -786,7 +786,7 @@
     <t>pmsr:INI1784603367388</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821935</t>
+    <t>pmsr:DPL1784614821935</t>
   </si>
   <si>
     <t>Portátil Workstation SN:030030 at UA Main Simulation Room</t>
@@ -795,7 +795,7 @@
     <t>pmsr:INI1784603367390</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821936</t>
+    <t>pmsr:DPL1784614821936</t>
   </si>
   <si>
     <t>Portátil Workstation SN:030031 at UA Main Simulation Room</t>
@@ -804,7 +804,7 @@
     <t>pmsr:INI1784603367391</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821937</t>
+    <t>pmsr:DPL1784614821937</t>
   </si>
   <si>
     <t>Projetor Video (suporte teto) SN:030032 at UA Main Simulation Room</t>
@@ -813,7 +813,7 @@
     <t>pmsr:INI1784603367392</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821938</t>
+    <t>pmsr:DPL1784614821938</t>
   </si>
   <si>
     <t>Simulador de adulto para o ensino de procedimentos fundamentais de cuidados de emergência SN:030033 at UA Main Simulation Room</t>
@@ -822,7 +822,7 @@
     <t>pmsr:INI1784603367394</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821939</t>
+    <t>pmsr:DPL1784614821939</t>
   </si>
   <si>
     <t>Simulador de Aparelho de Anestesia SN:030034 at UA Main Simulation Room</t>
@@ -831,7 +831,7 @@
     <t>pmsr:INI1784603367395</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821940</t>
+    <t>pmsr:DPL1784614821940</t>
   </si>
   <si>
     <t>Simulador de cuidados pediátricos SN:030035 at UA Main Simulation Room</t>
@@ -840,7 +840,7 @@
     <t>pmsr:INI1784603367396</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821941</t>
+    <t>pmsr:DPL1784614821941</t>
   </si>
   <si>
     <t>Simulador de Emergência, Trauma e SAV SN:030036 at UA Main Simulation Room</t>
@@ -849,7 +849,7 @@
     <t>pmsr:INI1784603367398</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821942</t>
+    <t>pmsr:DPL1784614821942</t>
   </si>
   <si>
     <t>Simulador de Ventilador SN:030037 at UA Main Simulation Room</t>
@@ -858,7 +858,7 @@
     <t>pmsr:INI1784603367399</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821943</t>
+    <t>pmsr:DPL1784614821943</t>
   </si>
   <si>
     <t>Small Rig Cage SN:030038 at UA Main Simulation Room</t>
@@ -867,7 +867,7 @@
     <t>pmsr:INI1784603367400</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821944</t>
+    <t>pmsr:DPL1784614821944</t>
   </si>
   <si>
     <t>Tripé Manfrotto SN:030039 at UA Main Simulation Room</t>
@@ -876,7 +876,7 @@
     <t>pmsr:INI1784603367402</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821945</t>
+    <t>pmsr:DPL1784614821945</t>
   </si>
   <si>
     <t>Ecógrafo portátil SN:040001 at IPB Main Simulation Room</t>
@@ -888,7 +888,7 @@
     <t>pmsr:INI1784603367403</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821946</t>
+    <t>pmsr:DPL1784614821946</t>
   </si>
   <si>
     <t>Espirómetro SN:040002 at IPB Main Simulation Room</t>
@@ -897,7 +897,7 @@
     <t>pmsr:INI1784603367404</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821947</t>
+    <t>pmsr:DPL1784614821947</t>
   </si>
   <si>
     <t>Localizador de veias por infravermelhos SN:040003 at IPB Main Simulation Room</t>
@@ -906,7 +906,7 @@
     <t>pmsr:INI1784603367406</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821948</t>
+    <t>pmsr:DPL1784614821948</t>
   </si>
   <si>
     <t>Localizador de veias por infravermelhos SN:040004 at IPB Main Simulation Room</t>
@@ -915,7 +915,7 @@
     <t>pmsr:INI1784603367407</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821949</t>
+    <t>pmsr:DPL1784614821949</t>
   </si>
   <si>
     <t>Mesa Body Interact SN:040005 at IPB Main Simulation Room</t>
@@ -924,7 +924,7 @@
     <t>pmsr:INI1784603367408</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821950</t>
+    <t>pmsr:DPL1784614821950</t>
   </si>
   <si>
     <t>Mesa de anatomia SN:040006 at IPB Main Simulation Room</t>
@@ -933,7 +933,7 @@
     <t>pmsr:INI1784603367410</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821951</t>
+    <t>pmsr:DPL1784614821951</t>
   </si>
   <si>
     <t>Modelo Dani SN:040007 at IPB Main Simulation Room</t>
@@ -942,7 +942,7 @@
     <t>pmsr:INI1784603367411</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821952</t>
+    <t>pmsr:DPL1784614821952</t>
   </si>
   <si>
     <t>Modelo Suporte Avançado de Vida SN:040008 at IPB Main Simulation Room</t>
@@ -951,7 +951,7 @@
     <t>pmsr:INI1784603367412</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821953</t>
+    <t>pmsr:DPL1784614821953</t>
   </si>
   <si>
     <t>Monitor Cardíaco de simulação SN:040009 at IPB Main Simulation Room</t>
@@ -960,7 +960,7 @@
     <t>pmsr:INI1784603367413</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821954</t>
+    <t>pmsr:DPL1784614821954</t>
   </si>
   <si>
     <t>Simulador de Ecografia SN:040010 at IPB Main Simulation Room</t>
@@ -969,7 +969,7 @@
     <t>pmsr:INI1784603367415</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821955</t>
+    <t>pmsr:DPL1784614821955</t>
   </si>
   <si>
     <t>Simulador de inserção de cateter central SN:040011 at IPB Main Simulation Room</t>
@@ -978,7 +978,7 @@
     <t>pmsr:INI1784603367416</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821956</t>
+    <t>pmsr:DPL1784614821956</t>
   </si>
   <si>
     <t>Simulador de inserção de PICC SN:040012 at IPB Main Simulation Room</t>
@@ -987,7 +987,7 @@
     <t>pmsr:INI1784603367417</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821957</t>
+    <t>pmsr:DPL1784614821957</t>
   </si>
   <si>
     <t>Simulador de sutura SN:040013 at IPB Main Simulation Room</t>
@@ -996,7 +996,7 @@
     <t>pmsr:INI1784603367419</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821958</t>
+    <t>pmsr:DPL1784614821958</t>
   </si>
   <si>
     <t>Simulador de via aérea difícil SN:040014 at IPB Main Simulation Room</t>
@@ -1005,7 +1005,7 @@
     <t>pmsr:INI1784603367420</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821959</t>
+    <t>pmsr:DPL1784614821959</t>
   </si>
   <si>
     <t>Simuladores de acesso vascular por ultrassom SN:040015 at IPB Main Simulation Room</t>
@@ -1014,7 +1014,7 @@
     <t>pmsr:INI1784603367421</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821960</t>
+    <t>pmsr:DPL1784614821960</t>
   </si>
   <si>
     <t>Torres de computadores SN:040016 at IPB Main Simulation Room</t>
@@ -1023,7 +1023,7 @@
     <t>pmsr:INI1784603367423</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821961</t>
+    <t>pmsr:DPL1784614821961</t>
   </si>
   <si>
     <t>Torres de computadores SN:040017 at IPB Main Simulation Room</t>
@@ -1032,7 +1032,7 @@
     <t>pmsr:INI1784603367424</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821962</t>
+    <t>pmsr:DPL1784614821962</t>
   </si>
   <si>
     <t>Torres de computadores SN:040018 at IPB Main Simulation Room</t>
@@ -1041,7 +1041,7 @@
     <t>pmsr:INI1784603367425</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821963</t>
+    <t>pmsr:DPL1784614821963</t>
   </si>
   <si>
     <t>Torres de computadores SN:040019 at IPB Main Simulation Room</t>
@@ -1050,7 +1050,7 @@
     <t>pmsr:INI1784603367427</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821964</t>
+    <t>pmsr:DPL1784614821964</t>
   </si>
   <si>
     <t>Torres de computadores SN:040020 at IPB Main Simulation Room</t>
@@ -1059,7 +1059,7 @@
     <t>pmsr:INI1784603367428</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821965</t>
+    <t>pmsr:DPL1784614821965</t>
   </si>
   <si>
     <t>Torres de computadores SN:040021 at IPB Main Simulation Room</t>
@@ -1068,7 +1068,7 @@
     <t>pmsr:INI1784603367429</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821966</t>
+    <t>pmsr:DPL1784614821966</t>
   </si>
   <si>
     <t>Torres de computadores SN:040022 at IPB Main Simulation Room</t>
@@ -1077,7 +1077,7 @@
     <t>pmsr:INI1784603367431</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821967</t>
+    <t>pmsr:DPL1784614821967</t>
   </si>
   <si>
     <t>Torres de computadores SN:040023 at IPB Main Simulation Room</t>
@@ -1086,7 +1086,7 @@
     <t>pmsr:INI1784603367432</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821968</t>
+    <t>pmsr:DPL1784614821968</t>
   </si>
   <si>
     <t>Torres de computadores SN:040024 at IPB Main Simulation Room</t>
@@ -1095,7 +1095,7 @@
     <t>pmsr:INI1784603367433</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821969</t>
+    <t>pmsr:DPL1784614821969</t>
   </si>
   <si>
     <t>Torres de computadores SN:040025 at IPB Main Simulation Room</t>
@@ -1104,7 +1104,7 @@
     <t>pmsr:INI1784603367434</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821970</t>
+    <t>pmsr:DPL1784614821970</t>
   </si>
   <si>
     <t>Torres de computadores SN:040026 at IPB Main Simulation Room</t>
@@ -1113,7 +1113,7 @@
     <t>pmsr:INI1784603367436</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821971</t>
+    <t>pmsr:DPL1784614821971</t>
   </si>
   <si>
     <t>Torres de computadores SN:040027 at IPB Main Simulation Room</t>
@@ -1122,7 +1122,7 @@
     <t>pmsr:INI1784603367437</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821972</t>
+    <t>pmsr:DPL1784614821972</t>
   </si>
   <si>
     <t>Torres de computadores SN:040028 at IPB Main Simulation Room</t>
@@ -1131,7 +1131,7 @@
     <t>pmsr:INI1784603367438</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821973</t>
+    <t>pmsr:DPL1784614821973</t>
   </si>
   <si>
     <t>Ecografo SN:050001 at IPVC Main Simulation Room</t>
@@ -1143,7 +1143,7 @@
     <t>pmsr:INI1784603367440</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821974</t>
+    <t>pmsr:DPL1784614821974</t>
   </si>
   <si>
     <t>Localizadores de veias infravermelhos SN:050002 at IPVC Main Simulation Room</t>
@@ -1152,7 +1152,7 @@
     <t>pmsr:INI1784603367441</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821975</t>
+    <t>pmsr:DPL1784614821975</t>
   </si>
   <si>
     <t>Membros para cateterismo SN:050003 at IPVC Main Simulation Room</t>
@@ -1161,7 +1161,7 @@
     <t>pmsr:INI1784603367442</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821976</t>
+    <t>pmsr:DPL1784614821976</t>
   </si>
   <si>
     <t>Membros para cateterismo SN:050004 at IPVC Main Simulation Room</t>
@@ -1170,7 +1170,7 @@
     <t>pmsr:INI1784603367444</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821977</t>
+    <t>pmsr:DPL1784614821977</t>
   </si>
   <si>
     <t>Simulador decisão clínica SN:050005 at IPVC Main Simulation Room</t>
@@ -1179,7 +1179,7 @@
     <t>pmsr:INI1784603367445</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821978</t>
+    <t>pmsr:DPL1784614821978</t>
   </si>
   <si>
     <t>Simulador Obstetrícia SN:050006 at IPVC Main Simulation Room</t>
@@ -1188,7 +1188,7 @@
     <t>pmsr:INI1784603367446</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821979</t>
+    <t>pmsr:DPL1784614821979</t>
   </si>
   <si>
     <t>Simulador pediátrico SN:050007 at IPVC Main Simulation Room</t>
@@ -1197,7 +1197,7 @@
     <t>pmsr:INI1784603367448</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821980</t>
+    <t>pmsr:DPL1784614821980</t>
   </si>
   <si>
     <t>Sistema de imagem e som (geral) SN:050008 at IPVC Main Simulation Room</t>
@@ -1206,7 +1206,7 @@
     <t>pmsr:INI1784603367449</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821981</t>
+    <t>pmsr:DPL1784614821981</t>
   </si>
   <si>
     <t>Delsys SN:060001 at ISAVE Main Simulation Room</t>
@@ -1218,7 +1218,7 @@
     <t>pmsr:INI1784603367450</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821982</t>
+    <t>pmsr:DPL1784614821982</t>
   </si>
   <si>
     <t>Double robotics- Hybrid classroom SN:060002 at ISAVE Main Simulation Room</t>
@@ -1227,7 +1227,7 @@
     <t>pmsr:INI1784603367452</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821983</t>
+    <t>pmsr:DPL1784614821983</t>
   </si>
   <si>
     <t>Simulador adulto SN:060003 at ISAVE Main Simulation Room</t>
@@ -1236,7 +1236,7 @@
     <t>pmsr:INI1784603367453</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821984</t>
+    <t>pmsr:DPL1784614821984</t>
   </si>
   <si>
     <t>Simulador Obstétrico SN:060004 at ISAVE Main Simulation Room</t>
@@ -1245,7 +1245,7 @@
     <t>pmsr:INI1784603367454</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821985</t>
+    <t>pmsr:DPL1784614821985</t>
   </si>
   <si>
     <t>Simulador Obstétrico SN:060005 at ISAVE Main Simulation Room</t>
@@ -1254,7 +1254,7 @@
     <t>pmsr:INI1784603367456</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821986</t>
+    <t>pmsr:DPL1784614821986</t>
   </si>
   <si>
     <t>Simulador Obstétrico SN:060006 at ISAVE Main Simulation Room</t>
@@ -1263,7 +1263,7 @@
     <t>pmsr:INI1784603367457</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821987</t>
+    <t>pmsr:DPL1784614821987</t>
   </si>
   <si>
     <t>Simulador Pediátrico de Emergência SN:060007 at ISAVE Main Simulation Room</t>
@@ -1272,7 +1272,7 @@
     <t>pmsr:INI1784603367458</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821988</t>
+    <t>pmsr:DPL1784614821988</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070001 at UCP Main Simulation Room</t>
@@ -1284,7 +1284,7 @@
     <t>pmsr:INI1784603367459</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821989</t>
+    <t>pmsr:DPL1784614821989</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070002 at UCP Main Simulation Room</t>
@@ -1293,7 +1293,7 @@
     <t>pmsr:INI1784603367461</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821990</t>
+    <t>pmsr:DPL1784614821990</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070003 at UCP Main Simulation Room</t>
@@ -1302,7 +1302,7 @@
     <t>pmsr:INI1784603367462</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821991</t>
+    <t>pmsr:DPL1784614821991</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070004 at UCP Main Simulation Room</t>
@@ -1311,7 +1311,7 @@
     <t>pmsr:INI1784603367463</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821992</t>
+    <t>pmsr:DPL1784614821992</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070005 at UCP Main Simulation Room</t>
@@ -1320,7 +1320,7 @@
     <t>pmsr:INI1784603367465</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821993</t>
+    <t>pmsr:DPL1784614821993</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070006 at UCP Main Simulation Room</t>
@@ -1329,7 +1329,7 @@
     <t>pmsr:INI1784603367466</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821994</t>
+    <t>pmsr:DPL1784614821994</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070007 at UCP Main Simulation Room</t>
@@ -1338,7 +1338,7 @@
     <t>pmsr:INI1784603367467</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821995</t>
+    <t>pmsr:DPL1784614821995</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070008 at UCP Main Simulation Room</t>
@@ -1347,7 +1347,7 @@
     <t>pmsr:INI1784603367469</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821996</t>
+    <t>pmsr:DPL1784614821996</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070009 at UCP Main Simulation Room</t>
@@ -1356,7 +1356,7 @@
     <t>pmsr:INI1784603367470</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821997</t>
+    <t>pmsr:DPL1784614821997</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070010 at UCP Main Simulation Room</t>
@@ -1365,7 +1365,7 @@
     <t>pmsr:INI1784603367471</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821998</t>
+    <t>pmsr:DPL1784614821998</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070011 at UCP Main Simulation Room</t>
@@ -1374,7 +1374,7 @@
     <t>pmsr:INI1784603367473</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614821999</t>
+    <t>pmsr:DPL1784614821999</t>
   </si>
   <si>
     <t>Abdominal Palpation Model Set Pregnangy and birth SN:070012 at UCP Main Simulation Room</t>
@@ -1383,7 +1383,7 @@
     <t>pmsr:INI1784603367474</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822000</t>
+    <t>pmsr:DPL1784614822000</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070013 at UCP Main Simulation Room</t>
@@ -1392,7 +1392,7 @@
     <t>pmsr:INI1784603367475</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822001</t>
+    <t>pmsr:DPL1784614822001</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070014 at UCP Main Simulation Room</t>
@@ -1401,7 +1401,7 @@
     <t>pmsr:INI1784603367476</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822002</t>
+    <t>pmsr:DPL1784614822002</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070015 at UCP Main Simulation Room</t>
@@ -1410,7 +1410,7 @@
     <t>pmsr:INI1784603367478</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822003</t>
+    <t>pmsr:DPL1784614822003</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070016 at UCP Main Simulation Room</t>
@@ -1419,7 +1419,7 @@
     <t>pmsr:INI1784603367479</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822004</t>
+    <t>pmsr:DPL1784614822004</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070017 at UCP Main Simulation Room</t>
@@ -1428,7 +1428,7 @@
     <t>pmsr:INI1784603367480</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822005</t>
+    <t>pmsr:DPL1784614822005</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070018 at UCP Main Simulation Room</t>
@@ -1437,7 +1437,7 @@
     <t>pmsr:INI1784603367482</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822006</t>
+    <t>pmsr:DPL1784614822006</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070019 at UCP Main Simulation Room</t>
@@ -1446,7 +1446,7 @@
     <t>pmsr:INI1784603367483</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822007</t>
+    <t>pmsr:DPL1784614822007</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070020 at UCP Main Simulation Room</t>
@@ -1455,7 +1455,7 @@
     <t>pmsr:INI1784603367484</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822008</t>
+    <t>pmsr:DPL1784614822008</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070021 at UCP Main Simulation Room</t>
@@ -1464,7 +1464,7 @@
     <t>pmsr:INI1784603367486</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822009</t>
+    <t>pmsr:DPL1784614822009</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070022 at UCP Main Simulation Room</t>
@@ -1473,7 +1473,7 @@
     <t>pmsr:INI1784603367487</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822010</t>
+    <t>pmsr:DPL1784614822010</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070023 at UCP Main Simulation Room</t>
@@ -1482,7 +1482,7 @@
     <t>pmsr:INI1784603367488</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822011</t>
+    <t>pmsr:DPL1784614822011</t>
   </si>
   <si>
     <t>Breast cancer palpation model SN:070024 at UCP Main Simulation Room</t>
@@ -1491,7 +1491,7 @@
     <t>pmsr:INI1784603367490</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822012</t>
+    <t>pmsr:DPL1784614822012</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070025 at UCP Main Simulation Room</t>
@@ -1500,7 +1500,7 @@
     <t>pmsr:INI1784603367491</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822013</t>
+    <t>pmsr:DPL1784614822013</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070026 at UCP Main Simulation Room</t>
@@ -1509,7 +1509,7 @@
     <t>pmsr:INI1784603367492</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822014</t>
+    <t>pmsr:DPL1784614822014</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070027 at UCP Main Simulation Room</t>
@@ -1518,7 +1518,7 @@
     <t>pmsr:INI1784603367494</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822015</t>
+    <t>pmsr:DPL1784614822015</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070028 at UCP Main Simulation Room</t>
@@ -1527,7 +1527,7 @@
     <t>pmsr:INI1784603367495</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822016</t>
+    <t>pmsr:DPL1784614822016</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070029 at UCP Main Simulation Room</t>
@@ -1536,7 +1536,7 @@
     <t>pmsr:INI1784603367496</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822017</t>
+    <t>pmsr:DPL1784614822017</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070030 at UCP Main Simulation Room</t>
@@ -1545,7 +1545,7 @@
     <t>pmsr:INI1784603367498</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822018</t>
+    <t>pmsr:DPL1784614822018</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070031 at UCP Main Simulation Room</t>
@@ -1554,7 +1554,7 @@
     <t>pmsr:INI1784603367499</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822019</t>
+    <t>pmsr:DPL1784614822019</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070032 at UCP Main Simulation Room</t>
@@ -1563,7 +1563,7 @@
     <t>pmsr:INI1784603367500</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822020</t>
+    <t>pmsr:DPL1784614822020</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070033 at UCP Main Simulation Room</t>
@@ -1572,7 +1572,7 @@
     <t>pmsr:INI1784603367502</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822021</t>
+    <t>pmsr:DPL1784614822021</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070034 at UCP Main Simulation Room</t>
@@ -1581,7 +1581,7 @@
     <t>pmsr:INI1784603367503</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822022</t>
+    <t>pmsr:DPL1784614822022</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070035 at UCP Main Simulation Room</t>
@@ -1590,7 +1590,7 @@
     <t>pmsr:INI1784603367504</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822023</t>
+    <t>pmsr:DPL1784614822023</t>
   </si>
   <si>
     <t>Breast examination simulator SN:070036 at UCP Main Simulation Room</t>
@@ -1599,7 +1599,7 @@
     <t>pmsr:INI1784603367506</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822024</t>
+    <t>pmsr:DPL1784614822024</t>
   </si>
   <si>
     <t>Butterfly IQ+ SN:070037 at UCP Main Simulation Room</t>
@@ -1608,7 +1608,7 @@
     <t>pmsr:INI1784603367507</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822025</t>
+    <t>pmsr:DPL1784614822025</t>
   </si>
   <si>
     <t>Butterfly IQ+ SN:070038 at UCP Main Simulation Room</t>
@@ -1617,7 +1617,7 @@
     <t>pmsr:INI1784603367508</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822026</t>
+    <t>pmsr:DPL1784614822026</t>
   </si>
   <si>
     <t>Butterfly IQ+ SN:070039 at UCP Main Simulation Room</t>
@@ -1626,7 +1626,7 @@
     <t>pmsr:INI1784603367509</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822027</t>
+    <t>pmsr:DPL1784614822027</t>
   </si>
   <si>
     <t>Butterfly IQ+ Pro education program SN:070040 at UCP Main Simulation Room</t>
@@ -1635,7 +1635,7 @@
     <t>pmsr:INI1784603367511</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822028</t>
+    <t>pmsr:DPL1784614822028</t>
   </si>
   <si>
     <t>Cabo Butterfly IQ+ SN:070041 at UCP Main Simulation Room</t>
@@ -1644,7 +1644,7 @@
     <t>pmsr:INI1784603367512</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822029</t>
+    <t>pmsr:DPL1784614822029</t>
   </si>
   <si>
     <t>Cabo Butterfly IQ+ SN:070042 at UCP Main Simulation Room</t>
@@ -1653,7 +1653,7 @@
     <t>pmsr:INI1784603367513</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822030</t>
+    <t>pmsr:DPL1784614822030</t>
   </si>
   <si>
     <t>Cabo Butterfly IQ+ SN:070043 at UCP Main Simulation Room</t>
@@ -1662,7 +1662,7 @@
     <t>pmsr:INI1784603367515</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822031</t>
+    <t>pmsr:DPL1784614822031</t>
   </si>
   <si>
     <t>Câmeras de Documentação Científica SN:070044 at UCP Main Simulation Room</t>
@@ -1671,7 +1671,7 @@
     <t>pmsr:INI1784603367516</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822032</t>
+    <t>pmsr:DPL1784614822032</t>
   </si>
   <si>
     <t>Câmeras de Documentação Científica SN:070045 at UCP Main Simulation Room</t>
@@ -1680,7 +1680,7 @@
     <t>pmsr:INI1784603367517</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822033</t>
+    <t>pmsr:DPL1784614822033</t>
   </si>
   <si>
     <t>Câmeras de Documentação Científica SN:070046 at UCP Main Simulation Room</t>
@@ -1689,7 +1689,7 @@
     <t>pmsr:INI1784603367519</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822034</t>
+    <t>pmsr:DPL1784614822034</t>
   </si>
   <si>
     <t>Câmeras de Documentação Científica SN:070047 at UCP Main Simulation Room</t>
@@ -1698,7 +1698,7 @@
     <t>pmsr:INI1784603367520</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822035</t>
+    <t>pmsr:DPL1784614822035</t>
   </si>
   <si>
     <t>Câmeras de Documentação Científica SN:070048 at UCP Main Simulation Room</t>
@@ -1707,7 +1707,7 @@
     <t>pmsr:INI1784603367521</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822036</t>
+    <t>pmsr:DPL1784614822036</t>
   </si>
   <si>
     <t>Desfibrilhador automático externo para SBV SN:070049 at UCP Main Simulation Room</t>
@@ -1716,7 +1716,7 @@
     <t>pmsr:INI1784603367523</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822037</t>
+    <t>pmsr:DPL1784614822037</t>
   </si>
   <si>
     <t>Desfibrilhador automático externo para SBV SN:070050 at UCP Main Simulation Room</t>
@@ -1725,7 +1725,7 @@
     <t>pmsr:INI1784603367524</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822038</t>
+    <t>pmsr:DPL1784614822038</t>
   </si>
   <si>
     <t>Injection trainer SN:070051 at UCP Main Simulation Room</t>
@@ -1734,7 +1734,7 @@
     <t>pmsr:INI1784603367525</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822039</t>
+    <t>pmsr:DPL1784614822039</t>
   </si>
   <si>
     <t>Injection trainer SN:070052 at UCP Main Simulation Room</t>
@@ -1743,7 +1743,7 @@
     <t>pmsr:INI1784603367527</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822040</t>
+    <t>pmsr:DPL1784614822040</t>
   </si>
   <si>
     <t>Injection trainer SN:070053 at UCP Main Simulation Room</t>
@@ -1752,7 +1752,7 @@
     <t>pmsr:INI1784603367528</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822041</t>
+    <t>pmsr:DPL1784614822041</t>
   </si>
   <si>
     <t>Injection trainer SN:070054 at UCP Main Simulation Room</t>
@@ -1761,7 +1761,7 @@
     <t>pmsr:INI1784603367529</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822042</t>
+    <t>pmsr:DPL1784614822042</t>
   </si>
   <si>
     <t>Injection trainer SN:070055 at UCP Main Simulation Room</t>
@@ -1770,7 +1770,7 @@
     <t>pmsr:INI1784603367531</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822043</t>
+    <t>pmsr:DPL1784614822043</t>
   </si>
   <si>
     <t>Injection trainer SN:070056 at UCP Main Simulation Room</t>
@@ -1779,7 +1779,7 @@
     <t>pmsr:INI1784603367532</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822044</t>
+    <t>pmsr:DPL1784614822044</t>
   </si>
   <si>
     <t>Injection trainer SN:070057 at UCP Main Simulation Room</t>
@@ -1788,7 +1788,7 @@
     <t>pmsr:INI1784603367533</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822045</t>
+    <t>pmsr:DPL1784614822045</t>
   </si>
   <si>
     <t>Injection trainer SN:070058 at UCP Main Simulation Room</t>
@@ -1797,7 +1797,7 @@
     <t>pmsr:INI1784603367535</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822046</t>
+    <t>pmsr:DPL1784614822046</t>
   </si>
   <si>
     <t>Injection trainer SN:070059 at UCP Main Simulation Room</t>
@@ -1806,7 +1806,7 @@
     <t>pmsr:INI1784603367536</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822047</t>
+    <t>pmsr:DPL1784614822047</t>
   </si>
   <si>
     <t>Injection trainer SN:070060 at UCP Main Simulation Room</t>
@@ -1815,7 +1815,7 @@
     <t>pmsr:INI1784603367537</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822048</t>
+    <t>pmsr:DPL1784614822048</t>
   </si>
   <si>
     <t>Injection trainer SN:070061 at UCP Main Simulation Room</t>
@@ -1824,7 +1824,7 @@
     <t>pmsr:INI1784603367539</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822049</t>
+    <t>pmsr:DPL1784614822049</t>
   </si>
   <si>
     <t>Injection trainer SN:070062 at UCP Main Simulation Room</t>
@@ -1833,7 +1833,7 @@
     <t>pmsr:INI1784603367540</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822050</t>
+    <t>pmsr:DPL1784614822050</t>
   </si>
   <si>
     <t>Mala para Butterfly IQ+ SN:070063 at UCP Main Simulation Room</t>
@@ -1842,7 +1842,7 @@
     <t>pmsr:INI1784603367541</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822051</t>
+    <t>pmsr:DPL1784614822051</t>
   </si>
   <si>
     <t>Mala para Butterfly IQ+ SN:070064 at UCP Main Simulation Room</t>
@@ -1851,7 +1851,7 @@
     <t>pmsr:INI1784603367543</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822052</t>
+    <t>pmsr:DPL1784614822052</t>
   </si>
   <si>
     <t>Mala para Butterfly IQ+ SN:070065 at UCP Main Simulation Room</t>
@@ -1860,7 +1860,7 @@
     <t>pmsr:INI1784603367544</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822053</t>
+    <t>pmsr:DPL1784614822053</t>
   </si>
   <si>
     <t>Male inguinal hernia anatomy model SN:070066 at UCP Main Simulation Room</t>
@@ -1869,7 +1869,7 @@
     <t>pmsr:INI1784603367546</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822054</t>
+    <t>pmsr:DPL1784614822054</t>
   </si>
   <si>
     <t>Male inguinal hernia anatomy model SN:070067 at UCP Main Simulation Room</t>
@@ -1878,7 +1878,7 @@
     <t>pmsr:INI1784603367547</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822055</t>
+    <t>pmsr:DPL1784614822055</t>
   </si>
   <si>
     <t>Male inguinal hernia anatomy model SN:070068 at UCP Main Simulation Room</t>
@@ -1887,7 +1887,7 @@
     <t>pmsr:INI1784603367548</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822056</t>
+    <t>pmsr:DPL1784614822056</t>
   </si>
   <si>
     <t>Manequim exame ginecológico (GYN/AID) SN:070069 at UCP Main Simulation Room</t>
@@ -1896,7 +1896,7 @@
     <t>pmsr:INI1784603367550</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822057</t>
+    <t>pmsr:DPL1784614822057</t>
   </si>
   <si>
     <t>Manequim exame ginecológico (GYN/AID) SN:070070 at UCP Main Simulation Room</t>
@@ -1905,7 +1905,7 @@
     <t>pmsr:INI1784603367551</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822058</t>
+    <t>pmsr:DPL1784614822058</t>
   </si>
   <si>
     <t>Manequim exame masculino (Zack) SN:070071 at UCP Main Simulation Room</t>
@@ -1914,7 +1914,7 @@
     <t>pmsr:INI1784603367552</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822059</t>
+    <t>pmsr:DPL1784614822059</t>
   </si>
   <si>
     <t>Manequim exame masculino (Zack) SN:070072 at UCP Main Simulation Room</t>
@@ -1923,7 +1923,7 @@
     <t>pmsr:INI1784603367554</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822060</t>
+    <t>pmsr:DPL1784614822060</t>
   </si>
   <si>
     <t>Manequim palpação abdominal SN:070073 at UCP Main Simulation Room</t>
@@ -1932,7 +1932,7 @@
     <t>pmsr:INI1784603367555</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822061</t>
+    <t>pmsr:DPL1784614822061</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070074 at UCP Main Simulation Room</t>
@@ -1941,7 +1941,7 @@
     <t>pmsr:INI1784603367556</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822062</t>
+    <t>pmsr:DPL1784614822062</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070075 at UCP Main Simulation Room</t>
@@ -1950,7 +1950,7 @@
     <t>pmsr:INI1784603367558</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822063</t>
+    <t>pmsr:DPL1784614822063</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070076 at UCP Main Simulation Room</t>
@@ -1959,7 +1959,7 @@
     <t>pmsr:INI1784603367559</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822064</t>
+    <t>pmsr:DPL1784614822064</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070077 at UCP Main Simulation Room</t>
@@ -1968,7 +1968,7 @@
     <t>pmsr:INI1784603367561</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822065</t>
+    <t>pmsr:DPL1784614822065</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070078 at UCP Main Simulation Room</t>
@@ -1977,7 +1977,7 @@
     <t>pmsr:INI1784603367562</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822066</t>
+    <t>pmsr:DPL1784614822066</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070079 at UCP Main Simulation Room</t>
@@ -1986,7 +1986,7 @@
     <t>pmsr:INI1784603367563</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822067</t>
+    <t>pmsr:DPL1784614822067</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070080 at UCP Main Simulation Room</t>
@@ -1995,7 +1995,7 @@
     <t>pmsr:INI1784603367565</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822068</t>
+    <t>pmsr:DPL1784614822068</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070081 at UCP Main Simulation Room</t>
@@ -2004,7 +2004,7 @@
     <t>pmsr:INI1784603367566</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822069</t>
+    <t>pmsr:DPL1784614822069</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070082 at UCP Main Simulation Room</t>
@@ -2013,7 +2013,7 @@
     <t>pmsr:INI1784603367567</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822070</t>
+    <t>pmsr:DPL1784614822070</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070083 at UCP Main Simulation Room</t>
@@ -2022,7 +2022,7 @@
     <t>pmsr:INI1784603367569</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822071</t>
+    <t>pmsr:DPL1784614822071</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070084 at UCP Main Simulation Room</t>
@@ -2031,7 +2031,7 @@
     <t>pmsr:INI1784603367570</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822072</t>
+    <t>pmsr:DPL1784614822072</t>
   </si>
   <si>
     <t>Manequim palpação mamária SN:070085 at UCP Main Simulation Room</t>
@@ -2040,7 +2040,7 @@
     <t>pmsr:INI1784603367571</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822073</t>
+    <t>pmsr:DPL1784614822073</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070086 at UCP Main Simulation Room</t>
@@ -2049,7 +2049,7 @@
     <t>pmsr:INI1784603367573</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822074</t>
+    <t>pmsr:DPL1784614822074</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070087 at UCP Main Simulation Room</t>
@@ -2058,7 +2058,7 @@
     <t>pmsr:INI1784603367574</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822075</t>
+    <t>pmsr:DPL1784614822075</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070088 at UCP Main Simulation Room</t>
@@ -2067,7 +2067,7 @@
     <t>pmsr:INI1784603367575</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822076</t>
+    <t>pmsr:DPL1784614822076</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070089 at UCP Main Simulation Room</t>
@@ -2076,7 +2076,7 @@
     <t>pmsr:INI1784603367577</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822077</t>
+    <t>pmsr:DPL1784614822077</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070090 at UCP Main Simulation Room</t>
@@ -2085,7 +2085,7 @@
     <t>pmsr:INI1784603367578</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822078</t>
+    <t>pmsr:DPL1784614822078</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070091 at UCP Main Simulation Room</t>
@@ -2094,7 +2094,7 @@
     <t>pmsr:INI1784603367579</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822079</t>
+    <t>pmsr:DPL1784614822079</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070092 at UCP Main Simulation Room</t>
@@ -2103,7 +2103,7 @@
     <t>pmsr:INI1784603367581</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822080</t>
+    <t>pmsr:DPL1784614822080</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070093 at UCP Main Simulation Room</t>
@@ -2112,7 +2112,7 @@
     <t>pmsr:INI1784603367582</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822081</t>
+    <t>pmsr:DPL1784614822081</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070094 at UCP Main Simulation Room</t>
@@ -2121,7 +2121,7 @@
     <t>pmsr:INI1784603367583</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822082</t>
+    <t>pmsr:DPL1784614822082</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070095 at UCP Main Simulation Room</t>
@@ -2130,7 +2130,7 @@
     <t>pmsr:INI1784603367584</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822083</t>
+    <t>pmsr:DPL1784614822083</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070096 at UCP Main Simulation Room</t>
@@ -2139,7 +2139,7 @@
     <t>pmsr:INI1784603367586</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822084</t>
+    <t>pmsr:DPL1784614822084</t>
   </si>
   <si>
     <t>Manequim punção intraossea SN:070097 at UCP Main Simulation Room</t>
@@ -2148,7 +2148,7 @@
     <t>pmsr:INI1784603367587</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822085</t>
+    <t>pmsr:DPL1784614822085</t>
   </si>
   <si>
     <t>Manequim simulador parto (Super OB Susie) SN:070098 at UCP Main Simulation Room</t>
@@ -2157,7 +2157,7 @@
     <t>pmsr:INI1784603367588</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822086</t>
+    <t>pmsr:DPL1784614822086</t>
   </si>
   <si>
     <t>Mesa de Anatomia Digital - Anatomage Table Convertible - Training - Protection - license and Handling SN:070099 at UCP Main Simulation Room</t>
@@ -2166,7 +2166,7 @@
     <t>pmsr:INI1784603367590</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822087</t>
+    <t>pmsr:DPL1784614822087</t>
   </si>
   <si>
     <t>Mesa de Anatomia Digital - Anatomage Table Convertible - Training - Protection - license and Handling SN:070100 at UCP Main Simulation Room</t>
@@ -2175,7 +2175,7 @@
     <t>pmsr:INI1784603367591</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822088</t>
+    <t>pmsr:DPL1784614822088</t>
   </si>
   <si>
     <t>Mesa de Anatomia Digital - Anatomage Table Convertible - Training - Protection - license and Handling SN:070101 at UCP Main Simulation Room</t>
@@ -2184,7 +2184,7 @@
     <t>pmsr:INI1784603367592</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822089</t>
+    <t>pmsr:DPL1784614822089</t>
   </si>
   <si>
     <t>Mesa de Anatomia Digital - Anatomage Table Convertible - Training - Protection - license and Handling SN:070102 at UCP Main Simulation Room</t>
@@ -2193,7 +2193,7 @@
     <t>pmsr:INI1784603367594</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822090</t>
+    <t>pmsr:DPL1784614822090</t>
   </si>
   <si>
     <t>Mesa de Anatomia Digital - Anatomage Table Convertible - Training - Protection - license and Handling SN:070103 at UCP Main Simulation Room</t>
@@ -2202,7 +2202,7 @@
     <t>pmsr:INI1784603367595</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822091</t>
+    <t>pmsr:DPL1784614822091</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070104 at UCP Main Simulation Room</t>
@@ -2211,7 +2211,7 @@
     <t>pmsr:INI1784603367596</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822092</t>
+    <t>pmsr:DPL1784614822092</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070105 at UCP Main Simulation Room</t>
@@ -2220,7 +2220,7 @@
     <t>pmsr:INI1784603367598</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822093</t>
+    <t>pmsr:DPL1784614822093</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070106 at UCP Main Simulation Room</t>
@@ -2229,7 +2229,7 @@
     <t>pmsr:INI1784603367599</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822094</t>
+    <t>pmsr:DPL1784614822094</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070107 at UCP Main Simulation Room</t>
@@ -2238,7 +2238,7 @@
     <t>pmsr:INI1784603367600</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822095</t>
+    <t>pmsr:DPL1784614822095</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070108 at UCP Main Simulation Room</t>
@@ -2247,7 +2247,7 @@
     <t>pmsr:INI1784603367602</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822096</t>
+    <t>pmsr:DPL1784614822096</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070109 at UCP Main Simulation Room</t>
@@ -2256,7 +2256,7 @@
     <t>pmsr:INI1784603367603</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822097</t>
+    <t>pmsr:DPL1784614822097</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070110 at UCP Main Simulation Room</t>
@@ -2265,7 +2265,7 @@
     <t>pmsr:INI1784603367604</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822098</t>
+    <t>pmsr:DPL1784614822098</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070111 at UCP Main Simulation Room</t>
@@ -2274,7 +2274,7 @@
     <t>pmsr:INI1784603367606</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822099</t>
+    <t>pmsr:DPL1784614822099</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070112 at UCP Main Simulation Room</t>
@@ -2283,7 +2283,7 @@
     <t>pmsr:INI1784603367607</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822100</t>
+    <t>pmsr:DPL1784614822100</t>
   </si>
   <si>
     <t>Microscópios Digitais SN:070113 at UCP Main Simulation Room</t>
@@ -2292,7 +2292,7 @@
     <t>pmsr:INI1784603367608</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822101</t>
+    <t>pmsr:DPL1784614822101</t>
   </si>
   <si>
     <t>Modelo da próstata SN:070114 at UCP Main Simulation Room</t>
@@ -2301,7 +2301,7 @@
     <t>pmsr:INI1784603367610</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822102</t>
+    <t>pmsr:DPL1784614822102</t>
   </si>
   <si>
     <t>Modelo da próstata SN:070115 at UCP Main Simulation Room</t>
@@ -2310,7 +2310,7 @@
     <t>pmsr:INI1784603367611</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822103</t>
+    <t>pmsr:DPL1784614822103</t>
   </si>
   <si>
     <t>Modelo da próstata SN:070116 at UCP Main Simulation Room</t>
@@ -2319,7 +2319,7 @@
     <t>pmsr:INI1784603367612</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822104</t>
+    <t>pmsr:DPL1784614822104</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070117 at UCP Main Simulation Room</t>
@@ -2328,7 +2328,7 @@
     <t>pmsr:INI1784603367614</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822105</t>
+    <t>pmsr:DPL1784614822105</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070118 at UCP Main Simulation Room</t>
@@ -2337,7 +2337,7 @@
     <t>pmsr:INI1784603367615</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822106</t>
+    <t>pmsr:DPL1784614822106</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070119 at UCP Main Simulation Room</t>
@@ -2346,7 +2346,7 @@
     <t>pmsr:INI1784603367616</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822107</t>
+    <t>pmsr:DPL1784614822107</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070120 at UCP Main Simulation Room</t>
@@ -2355,7 +2355,7 @@
     <t>pmsr:INI1784603367618</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822108</t>
+    <t>pmsr:DPL1784614822108</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070121 at UCP Main Simulation Room</t>
@@ -2364,7 +2364,7 @@
     <t>pmsr:INI1784603367619</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822109</t>
+    <t>pmsr:DPL1784614822109</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070122 at UCP Main Simulation Room</t>
@@ -2373,7 +2373,7 @@
     <t>pmsr:INI1784603367620</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822110</t>
+    <t>pmsr:DPL1784614822110</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070123 at UCP Main Simulation Room</t>
@@ -2382,7 +2382,7 @@
     <t>pmsr:INI1784603367622</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822111</t>
+    <t>pmsr:DPL1784614822111</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070124 at UCP Main Simulation Room</t>
@@ -2391,7 +2391,7 @@
     <t>pmsr:INI1784603367623</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822112</t>
+    <t>pmsr:DPL1784614822112</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070125 at UCP Main Simulation Room</t>
@@ -2400,7 +2400,7 @@
     <t>pmsr:INI1784603367624</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822113</t>
+    <t>pmsr:DPL1784614822113</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070126 at UCP Main Simulation Room</t>
@@ -2409,7 +2409,7 @@
     <t>pmsr:INI1784603367625</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822114</t>
+    <t>pmsr:DPL1784614822114</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070127 at UCP Main Simulation Room</t>
@@ -2418,7 +2418,7 @@
     <t>pmsr:INI1784603367627</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822115</t>
+    <t>pmsr:DPL1784614822115</t>
   </si>
   <si>
     <t>Pitting edema trainer SN:070128 at UCP Main Simulation Room</t>
@@ -2427,7 +2427,7 @@
     <t>pmsr:INI1784603367628</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822116</t>
+    <t>pmsr:DPL1784614822116</t>
   </si>
   <si>
     <t>Quadro Luminoso – Revolution Lightboard Studio Package SN:070129 at UCP Main Simulation Room</t>
@@ -2436,7 +2436,7 @@
     <t>pmsr:INI1784603367629</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822117</t>
+    <t>pmsr:DPL1784614822117</t>
   </si>
   <si>
     <t>Scanner ARTEC LEO SN:070130 at UCP Main Simulation Room</t>
@@ -2445,7 +2445,7 @@
     <t>pmsr:INI1784603367631</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822118</t>
+    <t>pmsr:DPL1784614822118</t>
   </si>
   <si>
     <t>Scanner ARTEC LEO SN:070131 at UCP Main Simulation Room</t>
@@ -2454,7 +2454,7 @@
     <t>pmsr:INI1784603367632</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822119</t>
+    <t>pmsr:DPL1784614822119</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070132 at UCP Main Simulation Room</t>
@@ -2463,7 +2463,7 @@
     <t>pmsr:INI1784603367633</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822120</t>
+    <t>pmsr:DPL1784614822120</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070133 at UCP Main Simulation Room</t>
@@ -2472,7 +2472,7 @@
     <t>pmsr:INI1784603367635</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822121</t>
+    <t>pmsr:DPL1784614822121</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070134 at UCP Main Simulation Room</t>
@@ -2481,7 +2481,7 @@
     <t>pmsr:INI1784603367636</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822122</t>
+    <t>pmsr:DPL1784614822122</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070135 at UCP Main Simulation Room</t>
@@ -2490,7 +2490,7 @@
     <t>pmsr:INI1784603367637</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822123</t>
+    <t>pmsr:DPL1784614822123</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070136 at UCP Main Simulation Room</t>
@@ -2499,7 +2499,7 @@
     <t>pmsr:INI1784603367639</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822124</t>
+    <t>pmsr:DPL1784614822124</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070137 at UCP Main Simulation Room</t>
@@ -2508,7 +2508,7 @@
     <t>pmsr:INI1784603367640</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822125</t>
+    <t>pmsr:DPL1784614822125</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070138 at UCP Main Simulation Room</t>
@@ -2517,7 +2517,7 @@
     <t>pmsr:INI1784603367641</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822126</t>
+    <t>pmsr:DPL1784614822126</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070139 at UCP Main Simulation Room</t>
@@ -2526,7 +2526,7 @@
     <t>pmsr:INI1784603367643</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822127</t>
+    <t>pmsr:DPL1784614822127</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070140 at UCP Main Simulation Room</t>
@@ -2535,7 +2535,7 @@
     <t>pmsr:INI1784603367644</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822128</t>
+    <t>pmsr:DPL1784614822128</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070141 at UCP Main Simulation Room</t>
@@ -2544,7 +2544,7 @@
     <t>pmsr:INI1784603367645</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822129</t>
+    <t>pmsr:DPL1784614822129</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070142 at UCP Main Simulation Room</t>
@@ -2553,7 +2553,7 @@
     <t>pmsr:INI1784603367647</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822130</t>
+    <t>pmsr:DPL1784614822130</t>
   </si>
   <si>
     <t>SimLeggings™ Pitting Edema SN:070143 at UCP Main Simulation Room</t>
@@ -2562,7 +2562,7 @@
     <t>pmsr:INI1784603367648</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822131</t>
+    <t>pmsr:DPL1784614822131</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070144 at UCP Main Simulation Room</t>
@@ -2571,7 +2571,7 @@
     <t>pmsr:INI1784603367649</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822132</t>
+    <t>pmsr:DPL1784614822132</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070145 at UCP Main Simulation Room</t>
@@ -2580,7 +2580,7 @@
     <t>pmsr:INI1784603367651</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822133</t>
+    <t>pmsr:DPL1784614822133</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070146 at UCP Main Simulation Room</t>
@@ -2589,7 +2589,7 @@
     <t>pmsr:INI1784603367652</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822134</t>
+    <t>pmsr:DPL1784614822134</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070147 at UCP Main Simulation Room</t>
@@ -2598,7 +2598,7 @@
     <t>pmsr:INI1784603367654</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822135</t>
+    <t>pmsr:DPL1784614822135</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070148 at UCP Main Simulation Room</t>
@@ -2607,7 +2607,7 @@
     <t>pmsr:INI1784603367655</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822136</t>
+    <t>pmsr:DPL1784614822136</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070149 at UCP Main Simulation Room</t>
@@ -2616,7 +2616,7 @@
     <t>pmsr:INI1784603367656</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822137</t>
+    <t>pmsr:DPL1784614822137</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070150 at UCP Main Simulation Room</t>
@@ -2625,7 +2625,7 @@
     <t>pmsr:INI1784603367657</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822138</t>
+    <t>pmsr:DPL1784614822138</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070151 at UCP Main Simulation Room</t>
@@ -2634,7 +2634,7 @@
     <t>pmsr:INI1784603367659</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822139</t>
+    <t>pmsr:DPL1784614822139</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070152 at UCP Main Simulation Room</t>
@@ -2643,7 +2643,7 @@
     <t>pmsr:INI1784603367660</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822140</t>
+    <t>pmsr:DPL1784614822140</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070153 at UCP Main Simulation Room</t>
@@ -2652,7 +2652,7 @@
     <t>pmsr:INI1784603367662</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822141</t>
+    <t>pmsr:DPL1784614822141</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070154 at UCP Main Simulation Room</t>
@@ -2661,7 +2661,7 @@
     <t>pmsr:INI1784603367663</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822142</t>
+    <t>pmsr:DPL1784614822142</t>
   </si>
   <si>
     <t>SimSleeves™ Lymphedema SN:070155 at UCP Main Simulation Room</t>
@@ -2670,7 +2670,7 @@
     <t>pmsr:INI1784603367664</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822143</t>
+    <t>pmsr:DPL1784614822143</t>
   </si>
   <si>
     <t>Simulador de doente adulto SN:070156 at UCP Main Simulation Room</t>
@@ -2679,7 +2679,7 @@
     <t>pmsr:INI1784603367666</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822144</t>
+    <t>pmsr:DPL1784614822144</t>
   </si>
   <si>
     <t>Simulador de doente geriátrico SN:070157 at UCP Main Simulation Room</t>
@@ -2688,7 +2688,7 @@
     <t>pmsr:INI1784603367667</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822145</t>
+    <t>pmsr:DPL1784614822145</t>
   </si>
   <si>
     <t>Simulador de doente oncológico SN:070158 at UCP Main Simulation Room</t>
@@ -2697,7 +2697,7 @@
     <t>pmsr:INI1784603367668</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822146</t>
+    <t>pmsr:DPL1784614822146</t>
   </si>
   <si>
     <t>Simulador de ecografia SN:070159 at UCP Main Simulation Room</t>
@@ -2706,7 +2706,7 @@
     <t>pmsr:INI1784603367670</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822147</t>
+    <t>pmsr:DPL1784614822147</t>
   </si>
   <si>
     <t>Simulador de toque rectal SN:070160 at UCP Main Simulation Room</t>
@@ -2715,7 +2715,7 @@
     <t>pmsr:INI1784603367671</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822148</t>
+    <t>pmsr:DPL1784614822148</t>
   </si>
   <si>
     <t>Simulador de toque rectal SN:070161 at UCP Main Simulation Room</t>
@@ -2724,7 +2724,7 @@
     <t>pmsr:INI1784603367672</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822149</t>
+    <t>pmsr:DPL1784614822149</t>
   </si>
   <si>
     <t>Simulador de toque rectal SN:070162 at UCP Main Simulation Room</t>
@@ -2733,7 +2733,7 @@
     <t>pmsr:INI1784603367673</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822150</t>
+    <t>pmsr:DPL1784614822150</t>
   </si>
   <si>
     <t>Simulador de toque rectal SN:070163 at UCP Main Simulation Room</t>
@@ -2742,7 +2742,7 @@
     <t>pmsr:INI1784603367675</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822151</t>
+    <t>pmsr:DPL1784614822151</t>
   </si>
   <si>
     <t>Simulador de toque rectal SN:070164 at UCP Main Simulation Room</t>
@@ -2751,7 +2751,7 @@
     <t>pmsr:INI1784603367676</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822152</t>
+    <t>pmsr:DPL1784614822152</t>
   </si>
   <si>
     <t>Simulador de toque rectal SN:070165 at UCP Main Simulation Room</t>
@@ -2760,7 +2760,7 @@
     <t>pmsr:INI1784603367677</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822153</t>
+    <t>pmsr:DPL1784614822153</t>
   </si>
   <si>
     <t>Simuladores de Hematologia SN:070166 at UCP Main Simulation Room</t>
@@ -2769,7 +2769,7 @@
     <t>pmsr:INI1784603367679</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822154</t>
+    <t>pmsr:DPL1784614822154</t>
   </si>
   <si>
     <t>Simuladores de Hematologia SN:070167 at UCP Main Simulation Room</t>
@@ -2778,7 +2778,7 @@
     <t>pmsr:INI1784603367680</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822155</t>
+    <t>pmsr:DPL1784614822155</t>
   </si>
   <si>
     <t>Simuladores de Hematologia SN:070168 at UCP Main Simulation Room</t>
@@ -2787,7 +2787,7 @@
     <t>pmsr:INI1784603367681</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822156</t>
+    <t>pmsr:DPL1784614822156</t>
   </si>
   <si>
     <t>Simuladores de Hematologia SN:070169 at UCP Main Simulation Room</t>
@@ -2796,7 +2796,7 @@
     <t>pmsr:INI1784603367683</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822157</t>
+    <t>pmsr:DPL1784614822157</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070170 at UCP Main Simulation Room</t>
@@ -2805,7 +2805,7 @@
     <t>pmsr:INI1784603367684</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822158</t>
+    <t>pmsr:DPL1784614822158</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070171 at UCP Main Simulation Room</t>
@@ -2814,7 +2814,7 @@
     <t>pmsr:INI1784603367685</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822159</t>
+    <t>pmsr:DPL1784614822159</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070172 at UCP Main Simulation Room</t>
@@ -2823,7 +2823,7 @@
     <t>pmsr:INI1784603367686</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822160</t>
+    <t>pmsr:DPL1784614822160</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070173 at UCP Main Simulation Room</t>
@@ -2832,7 +2832,7 @@
     <t>pmsr:INI1784603367688</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822161</t>
+    <t>pmsr:DPL1784614822161</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070174 at UCP Main Simulation Room</t>
@@ -2841,7 +2841,7 @@
     <t>pmsr:INI1784603367689</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822162</t>
+    <t>pmsr:DPL1784614822162</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070175 at UCP Main Simulation Room</t>
@@ -2850,7 +2850,7 @@
     <t>pmsr:INI1784603367690</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822163</t>
+    <t>pmsr:DPL1784614822163</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070176 at UCP Main Simulation Room</t>
@@ -2859,7 +2859,7 @@
     <t>pmsr:INI1784603367692</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822164</t>
+    <t>pmsr:DPL1784614822164</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070177 at UCP Main Simulation Room</t>
@@ -2868,7 +2868,7 @@
     <t>pmsr:INI1784603367693</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822165</t>
+    <t>pmsr:DPL1784614822165</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070178 at UCP Main Simulation Room</t>
@@ -2877,7 +2877,7 @@
     <t>pmsr:INI1784603367694</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822166</t>
+    <t>pmsr:DPL1784614822166</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070179 at UCP Main Simulation Room</t>
@@ -2886,7 +2886,7 @@
     <t>pmsr:INI1784603367696</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822167</t>
+    <t>pmsr:DPL1784614822167</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070180 at UCP Main Simulation Room</t>
@@ -2895,7 +2895,7 @@
     <t>pmsr:INI1784603367697</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822168</t>
+    <t>pmsr:DPL1784614822168</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070181 at UCP Main Simulation Room</t>
@@ -2904,7 +2904,7 @@
     <t>pmsr:INI1784603367698</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822169</t>
+    <t>pmsr:DPL1784614822169</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070182 at UCP Main Simulation Room</t>
@@ -2913,7 +2913,7 @@
     <t>pmsr:INI1784603367699</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822170</t>
+    <t>pmsr:DPL1784614822170</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070183 at UCP Main Simulation Room</t>
@@ -2922,7 +2922,7 @@
     <t>pmsr:INI1784603367701</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822171</t>
+    <t>pmsr:DPL1784614822171</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070184 at UCP Main Simulation Room</t>
@@ -2931,7 +2931,7 @@
     <t>pmsr:INI1784603367702</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822172</t>
+    <t>pmsr:DPL1784614822172</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070185 at UCP Main Simulation Room</t>
@@ -2940,7 +2940,7 @@
     <t>pmsr:INI1784603367703</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822173</t>
+    <t>pmsr:DPL1784614822173</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070186 at UCP Main Simulation Room</t>
@@ -2949,7 +2949,7 @@
     <t>pmsr:INI1784603367705</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822174</t>
+    <t>pmsr:DPL1784614822174</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070187 at UCP Main Simulation Room</t>
@@ -2958,7 +2958,7 @@
     <t>pmsr:INI1784603367706</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822175</t>
+    <t>pmsr:DPL1784614822175</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070188 at UCP Main Simulation Room</t>
@@ -2967,7 +2967,7 @@
     <t>pmsr:INI1784603367707</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822176</t>
+    <t>pmsr:DPL1784614822176</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070189 at UCP Main Simulation Room</t>
@@ -2976,7 +2976,7 @@
     <t>pmsr:INI1784603367709</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822177</t>
+    <t>pmsr:DPL1784614822177</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070190 at UCP Main Simulation Room</t>
@@ -2985,7 +2985,7 @@
     <t>pmsr:INI1784603367710</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822178</t>
+    <t>pmsr:DPL1784614822178</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070191 at UCP Main Simulation Room</t>
@@ -2994,7 +2994,7 @@
     <t>pmsr:INI1784603367711</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822179</t>
+    <t>pmsr:DPL1784614822179</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070192 at UCP Main Simulation Room</t>
@@ -3003,7 +3003,7 @@
     <t>pmsr:INI1784603367713</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822180</t>
+    <t>pmsr:DPL1784614822180</t>
   </si>
   <si>
     <t>Traje de envelhecimento e empatia SN:070193 at UCP Main Simulation Room</t>
@@ -3012,7 +3012,7 @@
     <t>pmsr:INI1784603367714</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822181</t>
+    <t>pmsr:DPL1784614822181</t>
   </si>
   <si>
     <t>Disfibrilhador Automático externo SN:070194 at UCP Main Simulation Room</t>
@@ -3021,7 +3021,7 @@
     <t>pmsr:INI1784603367715</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822182</t>
+    <t>pmsr:DPL1784614822182</t>
   </si>
   <si>
     <t>Ecógrafo estacionário Chison Cbit-9 SN:070195 at UCP Main Simulation Room</t>
@@ -3030,7 +3030,7 @@
     <t>pmsr:INI1784603367717</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822183</t>
+    <t>pmsr:DPL1784614822183</t>
   </si>
   <si>
     <t>Ecógrafo estacionário Chison Cbit-9 SN:070196 at UCP Main Simulation Room</t>
@@ -3039,7 +3039,7 @@
     <t>pmsr:INI1784603367718</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822184</t>
+    <t>pmsr:DPL1784614822184</t>
   </si>
   <si>
     <t>Eletroencefalógrafo (EEG) SN:070197 at UCP Main Simulation Room</t>
@@ -3048,7 +3048,7 @@
     <t>pmsr:INI1784603367719</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822185</t>
+    <t>pmsr:DPL1784614822185</t>
   </si>
   <si>
     <t>Eletroencefalógrafo (EEG) SN:070198 at UCP Main Simulation Room</t>
@@ -3057,7 +3057,7 @@
     <t>pmsr:INI1784603367721</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822186</t>
+    <t>pmsr:DPL1784614822186</t>
   </si>
   <si>
     <t>Motion Capture (requal) SN:070199 at UCP Main Simulation Room</t>
@@ -3066,7 +3066,7 @@
     <t>pmsr:INI1784603367722</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822187</t>
+    <t>pmsr:DPL1784614822187</t>
   </si>
   <si>
     <t>Scanner extra-oral SN:070200 at UCP Main Simulation Room</t>
@@ -3075,7 +3075,7 @@
     <t>pmsr:INI1784603367723</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822188</t>
+    <t>pmsr:DPL1784614822188</t>
   </si>
   <si>
     <t>Scanner intra-oral SN:070201 at UCP Main Simulation Room</t>
@@ -3084,7 +3084,7 @@
     <t>pmsr:INI1784603367725</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822189</t>
+    <t>pmsr:DPL1784614822189</t>
   </si>
   <si>
     <t>Simulador de Feridas SN:070202 at UCP Main Simulation Room</t>
@@ -3093,7 +3093,7 @@
     <t>pmsr:INI1784603367726</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822190</t>
+    <t>pmsr:DPL1784614822190</t>
   </si>
   <si>
     <t>Simulador de Feridas SN:070203 at UCP Main Simulation Room</t>
@@ -3102,7 +3102,7 @@
     <t>pmsr:INI1784603367727</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822191</t>
+    <t>pmsr:DPL1784614822191</t>
   </si>
   <si>
     <t>Simulador de Feridas SN:070204 at UCP Main Simulation Room</t>
@@ -3111,7 +3111,7 @@
     <t>pmsr:INI1784603367729</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822192</t>
+    <t>pmsr:DPL1784614822192</t>
   </si>
   <si>
     <t>Simulador Neonatal SN:070205 at UCP Main Simulation Room</t>
@@ -3120,7 +3120,7 @@
     <t>pmsr:INI1784603367730</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822193</t>
+    <t>pmsr:DPL1784614822193</t>
   </si>
   <si>
     <t>Simulador Obstétrico SN:070206 at UCP Main Simulation Room</t>
@@ -3129,7 +3129,7 @@
     <t>pmsr:INI1784603367731</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822194</t>
+    <t>pmsr:DPL1784614822194</t>
   </si>
   <si>
     <t>Sistema de desenho CAD SN:070207 at UCP Main Simulation Room</t>
@@ -3138,7 +3138,7 @@
     <t>pmsr:INI1784603367733</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822195</t>
+    <t>pmsr:DPL1784614822195</t>
   </si>
   <si>
     <t>Sistema de impressão 3D completo SN:070208 at UCP Main Simulation Room</t>
@@ -3147,7 +3147,7 @@
     <t>pmsr:INI1784603367734</t>
   </si>
   <si>
-    <t>pmsr:DEP1784614822196</t>
+    <t>pmsr:DPL1784614822196</t>
   </si>
   <si>
     <t>Sonda Periodontal Computorizada SN:070209 at UCP Main Simulation Room</t>
@@ -22488,7 +22488,7 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="11.1667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="24.6719" style="36" customWidth="1"/>
+    <col min="1" max="1" width="40.3047" style="36" customWidth="1"/>
     <col min="2" max="2" width="17.1719" style="36" customWidth="1"/>
     <col min="3" max="3" width="44.3516" style="36" customWidth="1"/>
     <col min="4" max="4" width="21.6719" style="36" customWidth="1"/>
@@ -22501,7 +22501,7 @@
     <col min="11" max="11" width="20" style="36" customWidth="1"/>
     <col min="12" max="12" width="23.8516" style="36" customWidth="1"/>
     <col min="13" max="13" width="31.1719" style="36" customWidth="1"/>
-    <col min="14" max="14" width="46.3281" style="36" customWidth="1"/>
+    <col min="14" max="14" width="46.3516" style="36" customWidth="1"/>
     <col min="15" max="26" width="8.85156" style="36" customWidth="1"/>
     <col min="27" max="16384" width="11.1719" style="36" customWidth="1"/>
   </cols>
@@ -50606,11 +50606,11 @@
   <cols>
     <col min="1" max="1" width="28.1719" style="37" customWidth="1"/>
     <col min="2" max="2" width="30" style="37" customWidth="1"/>
-    <col min="3" max="3" width="39.3516" style="37" customWidth="1"/>
+    <col min="3" max="3" width="82.6094" style="37" customWidth="1"/>
     <col min="4" max="4" width="21.1719" style="37" customWidth="1"/>
     <col min="5" max="5" width="12.8516" style="37" customWidth="1"/>
     <col min="6" max="6" width="12.5" style="37" customWidth="1"/>
-    <col min="7" max="7" width="43.9844" style="37" customWidth="1"/>
+    <col min="7" max="7" width="44" style="37" customWidth="1"/>
     <col min="8" max="26" width="8.85156" style="37" customWidth="1"/>
     <col min="27" max="16384" width="11.1719" style="37" customWidth="1"/>
   </cols>

</xml_diff>